<commit_message>
Repatriate xml escape and unescape functions
(Awaiting resolution of https://github.com/JuliaComputing/XML.jl/issues/53)
</commit_message>
<xml_diff>
--- a/data/escape.xlsx
+++ b/data/escape.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee85442dac9ca7a7/Documents/Julia/XLSX/XLSX.jl/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{FFD7FC4C-166E-4686-9EBB-879BC88BA5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E21AB69D-DEF9-458C-AFB2-B8B108AD8CFA}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{FFD7FC4C-166E-4686-9EBB-879BC88BA5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{041B9981-23C3-4DC8-BD7B-AB8C63EC84F4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="16665" yWindow="945" windowWidth="11775" windowHeight="10920" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="&amp; &amp; &quot; &gt; &lt; " sheetId="1" r:id="rId1"/>
@@ -36,80 +36,85 @@
     <t>&lt;&amp;&gt;</t>
   </si>
   <si>
-    <t>11&amp;amp;&amp;</t>
-  </si>
-  <si>
-    <t>21&amp;&amp;amp;&amp;&amp;</t>
-  </si>
-  <si>
-    <t>31&amp;&amp;&amp;amp;&amp;&amp;&amp;</t>
-  </si>
-  <si>
     <t>41&amp; &amp;; &amp;&amp;</t>
   </si>
   <si>
-    <t>12&amp;quot;&amp;</t>
-  </si>
-  <si>
-    <t>22&amp;&amp;quot;&amp;&amp;</t>
-  </si>
-  <si>
-    <t>32&amp;&amp;&amp;quot;&amp;&amp;&amp;</t>
-  </si>
-  <si>
     <t>42" "; ""</t>
   </si>
   <si>
-    <t>13&amp;lt;&amp;</t>
-  </si>
-  <si>
-    <t>23&amp;&amp;lt;&amp;&amp;</t>
-  </si>
-  <si>
-    <t>33&amp;&amp;&amp;lt;&amp;&amp;&amp;</t>
-  </si>
-  <si>
     <t>43&lt; &lt;; &lt;&lt;</t>
   </si>
   <si>
-    <t>14&amp;gt;&amp;</t>
-  </si>
-  <si>
-    <t>24&amp;&amp;gt;&amp;&amp;</t>
-  </si>
-  <si>
-    <t>34&amp;&amp;&amp;gt;&amp;&amp;&amp;</t>
-  </si>
-  <si>
     <t>44&gt; &gt;; &gt;&gt;</t>
   </si>
   <si>
-    <t>15&amp;apos;&amp;</t>
-  </si>
-  <si>
-    <t>25&amp;&amp;apos;&amp;&amp;</t>
-  </si>
-  <si>
-    <t>35&amp;&amp;&amp;apos;&amp;&amp;&amp;</t>
-  </si>
-  <si>
     <t>45' '; ''</t>
   </si>
   <si>
-    <t>&amp;&amp;apos; &amp;amp; &amp;quot; &amp;lt; &amp;gt; &amp;apos;</t>
+    <t>11&amp;&amp;</t>
+  </si>
+  <si>
+    <t>21&amp;&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>31&amp;&amp;&amp;&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>13&lt;&amp;</t>
+  </si>
+  <si>
+    <t>23&amp;&lt;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>33&amp;&amp;&lt;&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>14&gt;&amp;</t>
+  </si>
+  <si>
+    <t>24&amp;&gt;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>34&amp;&amp;&gt;&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>15'&amp;</t>
+  </si>
+  <si>
+    <t>25&amp;'&amp;&amp;</t>
+  </si>
+  <si>
+    <t>35&amp;&amp;'&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>&amp;' &amp; " &lt; &gt; '</t>
+  </si>
+  <si>
+    <t>32&amp;&amp;"&amp;&amp;&amp;</t>
+  </si>
+  <si>
+    <t>22&amp;"&amp;&amp;</t>
+  </si>
+  <si>
+    <t>12"&amp;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -132,8 +137,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,15 +462,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="13.25" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
@@ -471,30 +482,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -508,35 +519,35 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>